<commit_message>
Flor Alpuy Update Showroom Preventa 2026 2026-10-21 16:52:30
</commit_message>
<xml_diff>
--- a/cuotas preventa planes B.xlsx
+++ b/cuotas preventa planes B.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{98895067-F077-4204-A2EB-91DC349CC4BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FE486A-B246-431B-8CF2-E2BC453C9BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -538,7 +538,7 @@
     <col min="13" max="14" width="13.08984375" customWidth="1"/>
     <col min="15" max="15" width="12.36328125" customWidth="1"/>
     <col min="16" max="16" width="25.6328125" customWidth="1"/>
-    <col min="17" max="17" width="10.453125" customWidth="1"/>
+    <col min="17" max="17" width="45.1796875" customWidth="1"/>
     <col min="18" max="18" width="10.6328125" customWidth="1"/>
     <col min="19" max="20" width="18" customWidth="1"/>
     <col min="21" max="21" width="15.36328125" customWidth="1"/>

</xml_diff>